<commit_message>
🔒 [FULL] Daily chip data 2026-08-04 01:13
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-64/5d-140)&quot;;-0&quot; 億 (昨-64/5d-140)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +122億 &quot;&quot;(昨5/5d9)&quot;"/>
@@ -31,6 +31,7 @@
     <numFmt numFmtId="170" formatCode="0.0%"/>
     <numFmt numFmtId="171" formatCode="#,##0.0"/>
     <numFmt numFmtId="172" formatCode="#,##0.00;-#,##0.00"/>
+    <numFmt numFmtId="173" formatCode="0&quot; 檔 +120億 &quot;&quot;(昨5/5d9)&quot;"/>
   </numFmts>
   <fonts count="38">
     <font>
@@ -504,7 +505,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="194">
+  <cellXfs count="195">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -939,6 +940,9 @@
     <xf numFmtId="172" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="173" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1024,12 +1028,12 @@
     <comment ref="D18" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「張濬安(航海王)」獨佔比 83.1%
+領頭大戶「張濬安(航海王)」獨佔比 84.0%
   • 領頭金額 104,611 萬
-  • 合計淨買 125,848 萬
+  • 合計淨買 124,595 萬
   • 大戶數 12 位 (名義共識)
 判讀: 名義 12 位大戶共識,
-實質 1 人下注佔 83%,
+實質 1 人下注佔 84%,
 剩餘 11 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1037,9 +1041,9 @@
     <comment ref="D19" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 56.8%
-  • 領頭金額 55,828 萬
-  • 合計淨買 98,358 萬
+領頭大戶「陳族元」獨佔比 56.7%
+  • 領頭金額 55,645 萬
+  • 合計淨買 98,174 萬
   • 大戶數 13 位 (名義共識)
 判讀: 名義 13 位大戶共識,
 實質 1 人下注佔 57%,
@@ -1063,12 +1067,12 @@
     <comment ref="D21" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 57.9%
-  • 領頭金額 24,657 萬
-  • 合計淨買 42,552 萬
+領頭大戶「陳族元」獨佔比 58.8%
+  • 領頭金額 25,491 萬
+  • 合計淨買 43,385 萬
   • 大戶數 11 位 (名義共識)
 判讀: 名義 11 位大戶共識,
-實質 1 人下注佔 58%,
+實質 1 人下注佔 59%,
 剩餘 10 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1089,12 +1093,12 @@
     <comment ref="D23" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳律師」獨佔比 53.6%
+領頭大戶「陳律師」獨佔比 56.6%
   • 領頭金額 15,283 萬
-  • 合計淨買 28,538 萬
+  • 合計淨買 27,020 萬
   • 大戶數 12 位 (名義共識)
 判讀: 名義 12 位大戶共識,
-實質 1 人下注佔 54%,
+實質 1 人下注佔 57%,
 剩餘 11 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1450,7 +1454,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 📌 一般共識 2330 / 1303 / 2303 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 明日恐處置 6 檔: 3374/4542/4556...  |  訊號: 強偏多 (Q5 81.7%, hot=4)</t>
+          <t>💡 📌 一般共識 2330 / 1303 / 2303 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 明日恐處置 1 檔: 3362  |  訊號: 強偏多 (Q5 81.7%, hot=4)</t>
         </is>
       </c>
     </row>
@@ -1603,7 +1607,7 @@
         </is>
       </c>
       <c r="H15" s="17" t="n">
-        <v>193024</v>
+        <v>175305</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1625,7 +1629,7 @@
         <v>9</v>
       </c>
       <c r="N15" s="17" t="n">
-        <v>441946</v>
+        <v>424227</v>
       </c>
     </row>
     <row r="16">
@@ -1654,7 +1658,7 @@
         </is>
       </c>
       <c r="H16" s="17" t="n">
-        <v>85501</v>
+        <v>85215</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1676,7 +1680,7 @@
         <v>9</v>
       </c>
       <c r="N16" s="17" t="n">
-        <v>193870</v>
+        <v>193584</v>
       </c>
     </row>
     <row r="17">
@@ -1713,7 +1717,7 @@
         </is>
       </c>
       <c r="J17" s="18" t="n">
-        <v>52121</v>
+        <v>53420</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1727,7 +1731,7 @@
         <v>10</v>
       </c>
       <c r="N17" s="17" t="n">
-        <v>184850</v>
+        <v>186148</v>
       </c>
     </row>
     <row r="18">
@@ -1768,17 +1772,17 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="L18" s="18" t="n">
-        <v>3583</v>
+        <v>3049</v>
       </c>
       <c r="M18" s="19" t="n">
         <v>9</v>
       </c>
       <c r="N18" s="17" t="n">
-        <v>125848</v>
+        <v>124595</v>
       </c>
     </row>
     <row r="19">
@@ -1807,7 +1811,7 @@
         </is>
       </c>
       <c r="H19" s="17" t="n">
-        <v>55829</v>
+        <v>55645</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1829,7 +1833,7 @@
         <v>10</v>
       </c>
       <c r="N19" s="17" t="n">
-        <v>98358</v>
+        <v>98174</v>
       </c>
     </row>
     <row r="20">
@@ -1901,7 +1905,7 @@
         <v>11</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
@@ -1909,7 +1913,7 @@
         </is>
       </c>
       <c r="H21" s="17" t="n">
-        <v>24658</v>
+        <v>25491</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1931,7 +1935,7 @@
         <v>8</v>
       </c>
       <c r="N21" s="17" t="n">
-        <v>42552</v>
+        <v>43386</v>
       </c>
     </row>
     <row r="22">
@@ -2023,17 +2027,17 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>張濬安</t>
         </is>
       </c>
       <c r="L23" s="18" t="n">
-        <v>2399</v>
+        <v>1747</v>
       </c>
       <c r="M23" s="19" t="n">
         <v>9</v>
       </c>
       <c r="N23" s="17" t="n">
-        <v>28538</v>
+        <v>27020</v>
       </c>
     </row>
     <row r="24">
@@ -2109,7 +2113,7 @@
         </is>
       </c>
       <c r="G27" s="179" t="n">
-        <v>123.7623</v>
+        <v>123.95694</v>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
@@ -2118,7 +2122,7 @@
           <t>Q3 強共識股</t>
         </is>
       </c>
-      <c r="C28" s="180" t="n">
+      <c r="C28" s="194" t="n">
         <v>10</v>
       </c>
       <c r="F28" s="22" t="inlineStr">
@@ -2127,7 +2131,7 @@
         </is>
       </c>
       <c r="G28" s="181" t="n">
-        <v>0.2294531048392597</v>
+        <v>0.2292918916726649</v>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
@@ -2206,11 +2210,11 @@
         </is>
       </c>
       <c r="D34" s="33" t="n">
-        <v>1633313</v>
+        <v>1627932</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>27.7%</t>
+          <t>27.6%</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -2222,7 +2226,7 @@
         </is>
       </c>
       <c r="H34" s="33" t="n">
-        <v>441946</v>
+        <v>424227</v>
       </c>
       <c r="I34" s="183" t="n">
         <v>-0.0227</v>
@@ -2242,7 +2246,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>23.1%</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -2286,7 +2290,7 @@
         </is>
       </c>
       <c r="H36" s="33" t="n">
-        <v>231618</v>
+        <v>231704</v>
       </c>
       <c r="I36" s="184" t="n">
         <v>0.0495</v>
@@ -2318,7 +2322,7 @@
         </is>
       </c>
       <c r="H37" s="33" t="n">
-        <v>193870</v>
+        <v>193584</v>
       </c>
       <c r="I37" s="184" t="n">
         <v>0.0345</v>
@@ -2350,7 +2354,7 @@
         </is>
       </c>
       <c r="H38" s="33" t="n">
-        <v>184850</v>
+        <v>186148</v>
       </c>
       <c r="I38" s="183" t="n">
         <v>-0.0248</v>
@@ -2499,7 +2503,7 @@
         </is>
       </c>
       <c r="C51" s="33" t="n">
-        <v>1490209</v>
+        <v>1482753</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2507,7 +2511,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>200755</v>
+        <v>183670</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -2523,10 +2527,10 @@
         </is>
       </c>
       <c r="I51" s="33" t="n">
-        <v>127764</v>
+        <v>127776</v>
       </c>
       <c r="J51" s="185" t="n">
-        <v>0.3132101774207987</v>
+        <v>0.3032704561662108</v>
       </c>
     </row>
     <row r="52">
@@ -4087,7 +4091,7 @@
     <row r="34">
       <c r="C34" s="69" t="inlineStr">
         <is>
-          <t>明日恐處置 6 檔 (3374 / 4542 / 4556 ...)</t>
+          <t>明日恐處置 1 檔 (3362)</t>
         </is>
       </c>
     </row>
@@ -11799,31 +11803,31 @@
       </c>
       <c r="D190" s="110" t="inlineStr">
         <is>
-          <t>台積電(2330)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E190" s="111" t="n">
-        <v>83</v>
+        <v>328</v>
       </c>
       <c r="F190" s="111" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="G190" s="111" t="n">
-        <v>19834</v>
+        <v>13005</v>
       </c>
       <c r="H190" s="111" t="n">
-        <v>876</v>
+        <v>1903</v>
       </c>
       <c r="I190" s="111" t="n">
-        <v>18958</v>
+        <v>11102</v>
       </c>
       <c r="J190" s="112" t="n">
-        <v>2389.67</v>
+        <v>396.5</v>
       </c>
       <c r="K190" s="112" t="n">
-        <v>2190.25</v>
-      </c>
-      <c r="L190" s="192">
+        <v>396.5</v>
+      </c>
+      <c r="L190" s="191">
         <f>F190*(K190-J190)</f>
         <v/>
       </c>
@@ -11834,31 +11838,31 @@
       <c r="C191" s="113" t="n"/>
       <c r="D191" s="110" t="inlineStr">
         <is>
-          <t>南亞科(2408)</t>
+          <t>光寶科(2301)</t>
         </is>
       </c>
       <c r="E191" s="111" t="n">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="F191" s="111" t="n">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="G191" s="111" t="n">
-        <v>12447</v>
+        <v>7413</v>
       </c>
       <c r="H191" s="111" t="n">
-        <v>1912</v>
+        <v>69</v>
       </c>
       <c r="I191" s="111" t="n">
-        <v>10535</v>
+        <v>7344</v>
       </c>
       <c r="J191" s="112" t="n">
-        <v>379.49</v>
+        <v>229.5</v>
       </c>
       <c r="K191" s="112" t="n">
-        <v>398.33</v>
-      </c>
-      <c r="L191" s="191">
+        <v>229.33</v>
+      </c>
+      <c r="L191" s="192">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -11869,31 +11873,31 @@
       <c r="C192" s="113" t="n"/>
       <c r="D192" s="110" t="inlineStr">
         <is>
-          <t>光寶科(2301)</t>
+          <t>致茂(2360)</t>
         </is>
       </c>
       <c r="E192" s="111" t="n">
-        <v>323</v>
+        <v>21</v>
       </c>
       <c r="F192" s="111" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="G192" s="111" t="n">
-        <v>7413</v>
+        <v>4080</v>
       </c>
       <c r="H192" s="111" t="n">
-        <v>77</v>
+        <v>3246</v>
       </c>
       <c r="I192" s="111" t="n">
-        <v>7336</v>
+        <v>834</v>
       </c>
       <c r="J192" s="112" t="n">
-        <v>229.5</v>
+        <v>1942.62</v>
       </c>
       <c r="K192" s="112" t="n">
-        <v>257</v>
-      </c>
-      <c r="L192" s="191">
+        <v>1909.41</v>
+      </c>
+      <c r="L192" s="192">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -11904,31 +11908,31 @@
       <c r="C193" s="113" t="n"/>
       <c r="D193" s="110" t="inlineStr">
         <is>
-          <t>臻鼎-KY(4958)</t>
+          <t>聯電(2303)</t>
         </is>
       </c>
       <c r="E193" s="111" t="n">
-        <v>87</v>
+        <v>191</v>
       </c>
       <c r="F193" s="111" t="n">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="G193" s="111" t="n">
-        <v>3748</v>
+        <v>3892</v>
       </c>
       <c r="H193" s="111" t="n">
-        <v>1172</v>
+        <v>1098</v>
       </c>
       <c r="I193" s="111" t="n">
-        <v>2576</v>
+        <v>2794</v>
       </c>
       <c r="J193" s="112" t="n">
-        <v>430.8</v>
+        <v>203.74</v>
       </c>
       <c r="K193" s="112" t="n">
-        <v>433.96</v>
-      </c>
-      <c r="L193" s="191">
+        <v>171.62</v>
+      </c>
+      <c r="L193" s="192">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -11949,16 +11953,16 @@
         <v>1</v>
       </c>
       <c r="G194" s="111" t="n">
-        <v>3358</v>
+        <v>3401</v>
       </c>
       <c r="H194" s="111" t="n">
         <v>87</v>
       </c>
       <c r="I194" s="111" t="n">
-        <v>3271</v>
+        <v>3314</v>
       </c>
       <c r="J194" s="112" t="n">
-        <v>861</v>
+        <v>872</v>
       </c>
       <c r="K194" s="112" t="n">
         <v>872</v>
@@ -11974,29 +11978,29 @@
       <c r="C195" s="113" t="n"/>
       <c r="D195" s="110" t="inlineStr">
         <is>
-          <t>旺宏(2337)</t>
+          <t>台積電(2330)</t>
         </is>
       </c>
       <c r="E195" s="111" t="n">
-        <v>238</v>
+        <v>83</v>
       </c>
       <c r="F195" s="111" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="G195" s="111" t="n">
-        <v>2574</v>
+        <v>2749</v>
       </c>
       <c r="H195" s="111" t="n">
-        <v>351</v>
+        <v>1510</v>
       </c>
       <c r="I195" s="111" t="n">
-        <v>2223</v>
+        <v>1239</v>
       </c>
       <c r="J195" s="112" t="n">
-        <v>108.13</v>
+        <v>331.24</v>
       </c>
       <c r="K195" s="112" t="n">
-        <v>109.59</v>
+        <v>3775.5</v>
       </c>
       <c r="L195" s="191">
         <f>F195*(K195-J195)</f>
@@ -12009,29 +12013,29 @@
       <c r="C196" s="113" t="n"/>
       <c r="D196" s="110" t="inlineStr">
         <is>
-          <t>亞翔(6139)</t>
+          <t>台達電(2308)</t>
         </is>
       </c>
       <c r="E196" s="111" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F196" s="111" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G196" s="111" t="n">
-        <v>2266</v>
+        <v>2672</v>
       </c>
       <c r="H196" s="111" t="n">
-        <v>619</v>
+        <v>1617</v>
       </c>
       <c r="I196" s="111" t="n">
-        <v>1647</v>
+        <v>1055</v>
       </c>
       <c r="J196" s="112" t="n">
-        <v>755.23</v>
+        <v>1571.59</v>
       </c>
       <c r="K196" s="112" t="n">
-        <v>773.75</v>
+        <v>1617.3</v>
       </c>
       <c r="L196" s="191">
         <f>F196*(K196-J196)</f>
@@ -12044,29 +12048,29 @@
       <c r="C197" s="113" t="n"/>
       <c r="D197" s="110" t="inlineStr">
         <is>
-          <t>聯電(2303)</t>
+          <t>旺宏(2337)</t>
         </is>
       </c>
       <c r="E197" s="111" t="n">
-        <v>191</v>
+        <v>238</v>
       </c>
       <c r="F197" s="111" t="n">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="G197" s="111" t="n">
-        <v>2266</v>
+        <v>2630</v>
       </c>
       <c r="H197" s="111" t="n">
-        <v>771</v>
+        <v>354</v>
       </c>
       <c r="I197" s="111" t="n">
-        <v>1495</v>
+        <v>2276</v>
       </c>
       <c r="J197" s="112" t="n">
-        <v>118.62</v>
+        <v>110.5</v>
       </c>
       <c r="K197" s="112" t="n">
-        <v>120.5</v>
+        <v>110.5</v>
       </c>
       <c r="L197" s="191">
         <f>F197*(K197-J197)</f>
@@ -12079,29 +12083,29 @@
       <c r="C198" s="113" t="n"/>
       <c r="D198" s="110" t="inlineStr">
         <is>
-          <t>力積電(6770)</t>
+          <t>臻鼎-KY(4958)</t>
         </is>
       </c>
       <c r="E198" s="111" t="n">
-        <v>369</v>
+        <v>87</v>
       </c>
       <c r="F198" s="111" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="G198" s="111" t="n">
-        <v>2023</v>
+        <v>2445</v>
       </c>
       <c r="H198" s="111" t="n">
-        <v>88</v>
+        <v>1121</v>
       </c>
       <c r="I198" s="111" t="n">
-        <v>1935</v>
+        <v>1324</v>
       </c>
       <c r="J198" s="112" t="n">
-        <v>54.82</v>
+        <v>281</v>
       </c>
       <c r="K198" s="112" t="n">
-        <v>55.19</v>
+        <v>415.33</v>
       </c>
       <c r="L198" s="191">
         <f>F198*(K198-J198)</f>
@@ -12114,29 +12118,29 @@
       <c r="C199" s="113" t="n"/>
       <c r="D199" s="110" t="inlineStr">
         <is>
-          <t>文曄(3036)</t>
+          <t>穩懋(3105)</t>
         </is>
       </c>
       <c r="E199" s="111" t="n">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="F199" s="111" t="n">
-        <v>1</v>
+        <v>51</v>
       </c>
       <c r="G199" s="111" t="n">
-        <v>1974</v>
+        <v>2383</v>
       </c>
       <c r="H199" s="111" t="n">
-        <v>0</v>
+        <v>1576</v>
       </c>
       <c r="I199" s="111" t="n">
-        <v>1974</v>
+        <v>807</v>
       </c>
       <c r="J199" s="112" t="n">
-        <v>205.66</v>
+        <v>309.53</v>
       </c>
       <c r="K199" s="112" t="n">
-        <v>4</v>
+        <v>308.94</v>
       </c>
       <c r="L199" s="192">
         <f>F199*(K199-J199)</f>
@@ -22804,7 +22808,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="177" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-08-03 16:07 | 0/23 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-08-03 17:13 | 0/23 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-08-05 00:43
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="14">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-64/5d-140)&quot;;-0&quot; 億 (昨-64/5d-140)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +122億 &quot;&quot;(昨5/5d9)&quot;"/>
@@ -36,6 +36,7 @@
     <numFmt numFmtId="174" formatCode="+0&quot; 億 (昨+124/5d-85)&quot;;-0&quot; 億 (昨+124/5d-85)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="175" formatCode="0&quot; 檔 +78億 &quot;&quot;(昨10/5d9)&quot;"/>
     <numFmt numFmtId="176" formatCode="0.0%&quot; 市-1296億 &quot;&quot;(昨23/5d18)&quot;"/>
+    <numFmt numFmtId="177" formatCode="0.0%&quot; 市-1297億 &quot;&quot;(昨23/5d18)&quot;"/>
   </numFmts>
   <fonts count="39">
     <font>
@@ -515,7 +516,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="199">
+  <cellXfs count="200">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -963,6 +964,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1409,7 +1413,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 📌 一般共識 2330 / 2454 / 3711 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 除權息 19 檔: 00946, 00953B, 00985B ... | 明日恐處置 1 檔: 3362  |  訊號: 強偏多 (Q5 95%, hot=5)</t>
+          <t>💡 📌 一般共識 2330 / 2454 / 3711 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開: 今日無除權息+處置股  |  訊號: 強偏多 (Q5 95%, hot=5)</t>
         </is>
       </c>
     </row>
@@ -1962,23 +1966,23 @@
         <v>10</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
+          <t>陳律師</t>
+        </is>
+      </c>
+      <c r="H23" s="17" t="n">
+        <v>272</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
           <t>陳族元</t>
         </is>
       </c>
-      <c r="H23" s="17" t="n">
-        <v>293</v>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>陳律師</t>
-        </is>
-      </c>
       <c r="J23" s="18" t="n">
-        <v>272</v>
+        <v>223</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -1992,7 +1996,7 @@
         <v>7</v>
       </c>
       <c r="N23" s="17" t="n">
-        <v>1273</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -2017,7 +2021,7 @@
         </is>
       </c>
       <c r="G26" s="195" t="n">
-        <v>-89.31316</v>
+        <v>-90.55685</v>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
@@ -2034,8 +2038,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G27" s="197" t="n">
-        <v>0.1828725504138973</v>
+      <c r="G27" s="199" t="n">
+        <v>0.1824037584120599</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
@@ -2146,11 +2150,11 @@
         </is>
       </c>
       <c r="D34" s="33" t="n">
-        <v>1423998</v>
+        <v>1407222</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>26.6%</t>
+          <t>26.4%</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -2182,7 +2186,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>11.7%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -2584,11 +2588,11 @@
         <v>3</v>
       </c>
       <c r="E56" t="n">
-        <v>220750</v>
+        <v>212249</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>陳族元 連續 3 天加碼 3037 (累計 220,750 萬)</t>
+          <t>陳族元 連續 3 天加碼 3037 (累計 212,249 萬)</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2726,7 @@
         </is>
       </c>
       <c r="C63" s="33" t="n">
-        <v>1385934</v>
+        <v>1370793</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -2738,7 +2742,7 @@
         </is>
       </c>
       <c r="G63" s="33" t="n">
-        <v>118606</v>
+        <v>110105</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -2749,7 +2753,7 @@
         <v>97103</v>
       </c>
       <c r="J63" s="185" t="n">
-        <v>0.3400869954532483</v>
+        <v>0.3376421531186692</v>
       </c>
     </row>
     <row r="64">
@@ -3199,7 +3203,7 @@
     <row r="77" ht="22" customHeight="1">
       <c r="B77" s="54" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20260804)</t>
+          <t>▍ G. 注意股 (資料日 20260805)</t>
         </is>
       </c>
     </row>
@@ -3593,7 +3597,7 @@
     <row r="99" ht="22" customHeight="1">
       <c r="B99" s="65" t="inlineStr">
         <is>
-          <t>▍ I. 未來 30 天除權息 (有效 105 檔, 已剔除過期)</t>
+          <t>▍ I. 未來 30 天除權息 (有效 104 檔, 已剔除過期)</t>
         </is>
       </c>
     </row>
@@ -3627,17 +3631,17 @@
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260805</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>00946</t>
+          <t>00400A</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>群益科技高息成長</t>
+          <t>主動國泰動能高息</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -3646,23 +3650,23 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>0.058</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="102">
       <c r="B102" s="58" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260805</t>
         </is>
       </c>
       <c r="C102" s="58" t="inlineStr">
         <is>
-          <t>00953B</t>
+          <t>1437</t>
         </is>
       </c>
       <c r="D102" s="58" t="inlineStr">
         <is>
-          <t>群益優選非投等債</t>
+          <t>勤益控</t>
         </is>
       </c>
       <c r="E102" s="58" t="inlineStr">
@@ -3671,48 +3675,48 @@
         </is>
       </c>
       <c r="F102" s="58" t="n">
-        <v>0.061</v>
+        <v>0.481191</v>
       </c>
     </row>
     <row r="103">
       <c r="B103" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260805</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>00985B</t>
+          <t>1519</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>群益ESG投等債0-5</t>
+          <t>華城</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權息</t>
         </is>
       </c>
       <c r="F103" t="n">
-        <v>0.053</v>
+        <v>11</v>
       </c>
     </row>
     <row r="104">
       <c r="B104" s="58" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260805</t>
         </is>
       </c>
       <c r="C104" s="58" t="inlineStr">
         <is>
-          <t>1474</t>
+          <t>2427</t>
         </is>
       </c>
       <c r="D104" s="58" t="inlineStr">
         <is>
-          <t>弘裕</t>
+          <t>三商電</t>
         </is>
       </c>
       <c r="E104" s="58" t="inlineStr">
@@ -3721,73 +3725,73 @@
         </is>
       </c>
       <c r="F104" s="58" t="n">
-        <v>0.25</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260805</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>1736</t>
+          <t>2801</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>喬山</t>
+          <t>彰銀</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權息</t>
         </is>
       </c>
       <c r="F105" t="n">
-        <v>4.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="106">
       <c r="B106" s="58" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260805</t>
         </is>
       </c>
       <c r="C106" s="58" t="inlineStr">
         <is>
-          <t>2348</t>
+          <t>6201</t>
         </is>
       </c>
       <c r="D106" s="58" t="inlineStr">
         <is>
-          <t>海悅</t>
+          <t>亞弘電</t>
         </is>
       </c>
       <c r="E106" s="58" t="inlineStr">
         <is>
-          <t>權息</t>
+          <t>息</t>
         </is>
       </c>
       <c r="F106" s="58" t="n">
-        <v>5</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2348A</t>
+          <t>1419</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>海悅甲特</t>
+          <t>新紡</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -3796,23 +3800,23 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="108">
       <c r="B108" s="58" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C108" s="58" t="inlineStr">
         <is>
-          <t>2351</t>
+          <t>1439</t>
         </is>
       </c>
       <c r="D108" s="58" t="inlineStr">
         <is>
-          <t>順德</t>
+          <t>雋揚</t>
         </is>
       </c>
       <c r="E108" s="58" t="inlineStr">
@@ -3821,23 +3825,23 @@
         </is>
       </c>
       <c r="F108" s="58" t="n">
-        <v>1.028839</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2393</t>
+          <t>1713</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>億光</t>
+          <t>國化</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -3846,23 +3850,23 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>4.5</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="110">
       <c r="B110" s="58" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C110" s="58" t="inlineStr">
         <is>
-          <t>2543</t>
+          <t>2375</t>
         </is>
       </c>
       <c r="D110" s="58" t="inlineStr">
         <is>
-          <t>皇昌</t>
+          <t>凱美</t>
         </is>
       </c>
       <c r="E110" s="58" t="inlineStr">
@@ -3871,73 +3875,73 @@
         </is>
       </c>
       <c r="F110" s="58" t="n">
-        <v>1.027678</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2812</t>
+          <t>2762</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>台中銀</t>
+          <t>世界健身-KY</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>權息</t>
+          <t>息</t>
         </is>
       </c>
       <c r="F111" t="n">
-        <v>0.39</v>
+        <v>3.636991</v>
       </c>
     </row>
     <row r="112">
       <c r="B112" s="58" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C112" s="58" t="inlineStr">
         <is>
-          <t>2834</t>
+          <t>3003</t>
         </is>
       </c>
       <c r="D112" s="58" t="inlineStr">
         <is>
-          <t>臺企銀</t>
+          <t>健和興</t>
         </is>
       </c>
       <c r="E112" s="58" t="inlineStr">
         <is>
-          <t>權息</t>
+          <t>息</t>
         </is>
       </c>
       <c r="F112" s="58" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113">
       <c r="B113" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>3533</t>
+          <t>3033</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>嘉澤</t>
+          <t>威健</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -3946,23 +3950,23 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>34.93436</v>
+        <v>1.919856</v>
       </c>
     </row>
     <row r="114">
       <c r="B114" s="58" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C114" s="58" t="inlineStr">
         <is>
-          <t>3545</t>
+          <t>3376</t>
         </is>
       </c>
       <c r="D114" s="58" t="inlineStr">
         <is>
-          <t>敦泰</t>
+          <t>新日興</t>
         </is>
       </c>
       <c r="E114" s="58" t="inlineStr">
@@ -3971,23 +3975,23 @@
         </is>
       </c>
       <c r="F114" s="58" t="n">
-        <v>0.81494</v>
+        <v>3.999665</v>
       </c>
     </row>
     <row r="115">
       <c r="B115" t="inlineStr">
         <is>
-          <t>20260804</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>4190</t>
+          <t>5288</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>佐登-KY</t>
+          <t>豐祥-KY</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -3996,7 +4000,7 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>0.499953</v>
+        <v>6.502918</v>
       </c>
     </row>
   </sheetData>
@@ -4290,16 +4294,16 @@
       </c>
     </row>
     <row r="29">
-      <c r="C29" s="69" t="inlineStr">
-        <is>
-          <t>除權息 19 檔 (00946 / 00953B / 00985B ...)</t>
+      <c r="C29" s="71" t="inlineStr">
+        <is>
+          <t>今日無除權息</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="C30" s="69" t="inlineStr">
-        <is>
-          <t>明日恐處置 1 檔 (3362)</t>
+      <c r="C30" s="71" t="inlineStr">
+        <is>
+          <t>今日無處置股</t>
         </is>
       </c>
     </row>
@@ -4313,7 +4317,7 @@
     <row r="33" ht="22" customHeight="1">
       <c r="C33" s="198" t="inlineStr">
         <is>
-          <t>-89 億 淨買</t>
+          <t>-91 億 淨買</t>
         </is>
       </c>
     </row>
@@ -4437,7 +4441,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="B3" s="76" t="inlineStr">
         <is>
-          <t>大牌分析師 近 3/3 交易日出手 136 次 (111 檔), 風格分布: 隔日沖近似 25% / 當沖 17% / 留倉 57%, 漲停命中 11% (其中 🔒鎖漲停 8%), 前 5 大集中 32%, ⚠️ 處置股部位 2% (5 檔)。 主軸: 高頻交易。</t>
+          <t>大牌分析師 近 3/3 交易日出手 136 次 (111 檔), 風格分布: 隔日沖近似 25% / 當沖 17% / 留倉 57%, 漲停命中 11% (其中 🔒鎖漲停 8%), 前 5 大集中 32%, ⚠️ 處置股部位 2% (4 檔)。 主軸: 高頻交易。</t>
         </is>
       </c>
     </row>
@@ -12085,7 +12089,7 @@
         </is>
       </c>
       <c r="E192" s="111" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F192" s="111" t="n">
         <v>1</v>
@@ -12100,7 +12104,7 @@
         <v>12434</v>
       </c>
       <c r="J192" s="112" t="n">
-        <v>1027.77</v>
+        <v>1019.34</v>
       </c>
       <c r="K192" s="112" t="n">
         <v>25</v>
@@ -12155,10 +12159,10 @@
         </is>
       </c>
       <c r="E194" s="111" t="n">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="F194" s="111" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G194" s="111" t="n">
         <v>10447</v>
@@ -12170,12 +12174,12 @@
         <v>4615</v>
       </c>
       <c r="J194" s="112" t="n">
-        <v>435.31</v>
+        <v>414.58</v>
       </c>
       <c r="K194" s="112" t="n">
-        <v>435.25</v>
-      </c>
-      <c r="L194" s="192">
+        <v>428.85</v>
+      </c>
+      <c r="L194" s="191">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -12186,31 +12190,31 @@
       <c r="C195" s="113" t="n"/>
       <c r="D195" s="110" t="inlineStr">
         <is>
-          <t>欣興(3037)</t>
+          <t>貿聯-KY(3665)</t>
         </is>
       </c>
       <c r="E195" s="111" t="n">
-        <v>92</v>
+        <v>21</v>
       </c>
       <c r="F195" s="111" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="G195" s="111" t="n">
-        <v>8501</v>
+        <v>4752</v>
       </c>
       <c r="H195" s="111" t="n">
-        <v>3049</v>
+        <v>54</v>
       </c>
       <c r="I195" s="111" t="n">
-        <v>5452</v>
+        <v>4698</v>
       </c>
       <c r="J195" s="112" t="n">
-        <v>924</v>
+        <v>2263.1</v>
       </c>
       <c r="K195" s="112" t="n">
-        <v>924</v>
-      </c>
-      <c r="L195" s="191">
+        <v>538</v>
+      </c>
+      <c r="L195" s="192">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -12221,29 +12225,29 @@
       <c r="C196" s="113" t="n"/>
       <c r="D196" s="110" t="inlineStr">
         <is>
-          <t>貿聯-KY(3665)</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="E196" s="111" t="n">
-        <v>21</v>
+        <v>65</v>
       </c>
       <c r="F196" s="111" t="n">
-        <v>1</v>
+        <v>53</v>
       </c>
       <c r="G196" s="111" t="n">
-        <v>4752</v>
+        <v>3676</v>
       </c>
       <c r="H196" s="111" t="n">
-        <v>54</v>
+        <v>2996</v>
       </c>
       <c r="I196" s="111" t="n">
-        <v>4698</v>
+        <v>680</v>
       </c>
       <c r="J196" s="112" t="n">
-        <v>2263.1</v>
+        <v>565.5700000000001</v>
       </c>
       <c r="K196" s="112" t="n">
-        <v>538</v>
+        <v>565.1900000000001</v>
       </c>
       <c r="L196" s="192">
         <f>F196*(K196-J196)</f>
@@ -12256,31 +12260,31 @@
       <c r="C197" s="113" t="n"/>
       <c r="D197" s="110" t="inlineStr">
         <is>
-          <t>國巨*(2327)</t>
+          <t>日月光投控(3711)</t>
         </is>
       </c>
       <c r="E197" s="111" t="n">
-        <v>138</v>
+        <v>48</v>
       </c>
       <c r="F197" s="111" t="n">
-        <v>59</v>
+        <v>4</v>
       </c>
       <c r="G197" s="111" t="n">
-        <v>3676</v>
+        <v>2813</v>
       </c>
       <c r="H197" s="111" t="n">
-        <v>2996</v>
+        <v>233</v>
       </c>
       <c r="I197" s="111" t="n">
-        <v>680</v>
+        <v>2580</v>
       </c>
       <c r="J197" s="112" t="n">
-        <v>266.39</v>
+        <v>585.98</v>
       </c>
       <c r="K197" s="112" t="n">
-        <v>507.71</v>
-      </c>
-      <c r="L197" s="191">
+        <v>582</v>
+      </c>
+      <c r="L197" s="192">
         <f>F197*(K197-J197)</f>
         <v/>
       </c>
@@ -12291,29 +12295,29 @@
       <c r="C198" s="113" t="n"/>
       <c r="D198" s="110" t="inlineStr">
         <is>
-          <t>聯電(2303)</t>
+          <t>南亞(1303)</t>
         </is>
       </c>
       <c r="E198" s="111" t="n">
-        <v>244</v>
+        <v>141</v>
       </c>
       <c r="F198" s="111" t="n">
-        <v>47</v>
+        <v>85</v>
       </c>
       <c r="G198" s="111" t="n">
-        <v>2891</v>
+        <v>2410</v>
       </c>
       <c r="H198" s="111" t="n">
-        <v>557</v>
+        <v>1457</v>
       </c>
       <c r="I198" s="111" t="n">
-        <v>2334</v>
+        <v>953</v>
       </c>
       <c r="J198" s="112" t="n">
-        <v>118.5</v>
+        <v>170.89</v>
       </c>
       <c r="K198" s="112" t="n">
-        <v>118.51</v>
+        <v>171.36</v>
       </c>
       <c r="L198" s="191">
         <f>F198*(K198-J198)</f>
@@ -12326,31 +12330,31 @@
       <c r="C199" s="113" t="n"/>
       <c r="D199" s="110" t="inlineStr">
         <is>
-          <t>日月光投控(3711)</t>
+          <t>勤誠(8210)</t>
         </is>
       </c>
       <c r="E199" s="111" t="n">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="F199" s="111" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G199" s="111" t="n">
-        <v>2813</v>
+        <v>2256</v>
       </c>
       <c r="H199" s="111" t="n">
-        <v>233</v>
+        <v>574</v>
       </c>
       <c r="I199" s="111" t="n">
-        <v>2580</v>
+        <v>1682</v>
       </c>
       <c r="J199" s="112" t="n">
-        <v>585.98</v>
+        <v>1127.9</v>
       </c>
       <c r="K199" s="112" t="n">
-        <v>582</v>
-      </c>
-      <c r="L199" s="192">
+        <v>1147.4</v>
+      </c>
+      <c r="L199" s="191">
         <f>F199*(K199-J199)</f>
         <v/>
       </c>
@@ -23062,7 +23066,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="177" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-08-04 15:52 | 0/24 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-08-04 16:43 | 0/24 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-08-06 00:33
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -23,7 +23,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="17">
+  <numFmts count="18">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-64/5d-140)&quot;;-0&quot; 億 (昨-64/5d-140)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +122億 &quot;&quot;(昨5/5d9)&quot;"/>
@@ -41,6 +41,7 @@
     <numFmt numFmtId="178" formatCode="+0&quot; 億 (昨-91/5d-59)&quot;;-0&quot; 億 (昨-91/5d-59)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="179" formatCode="0&quot; 檔 +63億 &quot;&quot;(昨9/5d8)&quot;"/>
     <numFmt numFmtId="180" formatCode="0.0%&quot; 市-482億 &quot;&quot;(昨18/5d18)&quot;"/>
+    <numFmt numFmtId="181" formatCode="0.0%&quot; 市-475億 &quot;&quot;(昨18/5d18)&quot;"/>
   </numFmts>
   <fonts count="39">
     <font>
@@ -520,7 +521,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="204">
+  <cellXfs count="205">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -981,6 +982,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="181" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1066,12 +1070,12 @@
     <comment ref="D15" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「張濬安(航海王)」獨佔比 60.9%
+領頭大戶「張濬安(航海王)」獨佔比 60.3%
   • 領頭金額 136,742 萬
-  • 合計淨買 224,645 萬
+  • 合計淨買 226,692 萬
   • 大戶數 10 位 (名義共識)
 判讀: 名義 10 位大戶共識,
-實質 1 人下注佔 61%,
+實質 1 人下注佔 60%,
 剩餘 9 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1585,7 +1589,7 @@
         <v>10</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
@@ -1601,7 +1605,7 @@
         </is>
       </c>
       <c r="J15" s="18" t="n">
-        <v>56060</v>
+        <v>58107</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1615,7 +1619,7 @@
         <v>7</v>
       </c>
       <c r="N15" s="17" t="n">
-        <v>224645</v>
+        <v>226692</v>
       </c>
     </row>
     <row r="16">
@@ -1993,7 +1997,7 @@
         <v>11</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
@@ -2001,7 +2005,7 @@
         </is>
       </c>
       <c r="H23" s="17" t="n">
-        <v>5060</v>
+        <v>4888</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -2023,7 +2027,7 @@
         <v>8</v>
       </c>
       <c r="N23" s="17" t="n">
-        <v>19002</v>
+        <v>18830</v>
       </c>
     </row>
     <row r="24">
@@ -2146,7 +2150,7 @@
         <v>10</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G26" s="16" t="inlineStr">
         <is>
@@ -2176,7 +2180,7 @@
         <v>7</v>
       </c>
       <c r="N26" s="17" t="n">
-        <v>7730</v>
+        <v>7848</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
@@ -2201,7 +2205,7 @@
         </is>
       </c>
       <c r="G29" s="200" t="n">
-        <v>-187.38063</v>
+        <v>-183.99805</v>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
@@ -2218,8 +2222,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G30" s="202" t="n">
-        <v>0.1591557297445387</v>
+      <c r="G30" s="204" t="n">
+        <v>0.1595358900128013</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
@@ -2302,7 +2306,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>35.6%</t>
+          <t>35.5%</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2330,11 +2334,11 @@
         </is>
       </c>
       <c r="D37" s="33" t="n">
-        <v>1489607</v>
+        <v>1509116</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>26.8%</t>
+          <t>27.0%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2346,7 +2350,7 @@
         </is>
       </c>
       <c r="H37" s="33" t="n">
-        <v>224645</v>
+        <v>226692</v>
       </c>
       <c r="I37" s="184" t="n">
         <v>0.0206</v>
@@ -2738,18 +2742,18 @@
       </c>
       <c r="C58" s="58" t="inlineStr">
         <is>
-          <t>2383</t>
+          <t>1303</t>
         </is>
       </c>
       <c r="D58" s="58" t="n">
         <v>4</v>
       </c>
       <c r="E58" s="58" t="n">
-        <v>230495</v>
+        <v>232315</v>
       </c>
       <c r="F58" s="58" t="inlineStr">
         <is>
-          <t>陳族元 連續 4 天加碼 2383 (累計 230,495 萬)</t>
+          <t>陳族元 連續 4 天加碼 1303 (累計 232,315 萬)</t>
         </is>
       </c>
     </row>
@@ -2761,18 +2765,18 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>3653</t>
+          <t>2383</t>
         </is>
       </c>
       <c r="D59" t="n">
         <v>4</v>
       </c>
       <c r="E59" t="n">
-        <v>228922</v>
+        <v>230495</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>陳族元 連續 4 天加碼 3653 (累計 228,922 萬)</t>
+          <t>陳族元 連續 4 天加碼 2383 (累計 230,495 萬)</t>
         </is>
       </c>
     </row>
@@ -2784,18 +2788,18 @@
       </c>
       <c r="C60" s="58" t="inlineStr">
         <is>
-          <t>1303</t>
+          <t>3653</t>
         </is>
       </c>
       <c r="D60" s="58" t="n">
         <v>4</v>
       </c>
       <c r="E60" s="58" t="n">
-        <v>219005</v>
+        <v>228922</v>
       </c>
       <c r="F60" s="58" t="inlineStr">
         <is>
-          <t>陳族元 連續 4 天加碼 1303 (累計 219,005 萬)</t>
+          <t>陳族元 連續 4 天加碼 3653 (累計 228,922 萬)</t>
         </is>
       </c>
     </row>
@@ -2943,7 +2947,7 @@
         </is>
       </c>
       <c r="C67" s="33" t="n">
-        <v>1371660</v>
+        <v>1389992</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -2970,7 +2974,7 @@
         <v>124487</v>
       </c>
       <c r="J67" s="185" t="n">
-        <v>0.3274504853571938</v>
+        <v>0.3231317667636168</v>
       </c>
     </row>
     <row r="68">
@@ -4516,7 +4520,7 @@
     <row r="36" ht="22" customHeight="1">
       <c r="C36" s="198" t="inlineStr">
         <is>
-          <t>-187 億 淨買</t>
+          <t>-184 億 淨買</t>
         </is>
       </c>
     </row>
@@ -12249,31 +12253,31 @@
       <c r="C191" s="113" t="n"/>
       <c r="D191" s="110" t="inlineStr">
         <is>
-          <t>聯電(2303)</t>
+          <t>南亞(1303)</t>
         </is>
       </c>
       <c r="E191" s="111" t="n">
-        <v>696</v>
+        <v>752</v>
       </c>
       <c r="F191" s="111" t="n">
-        <v>133</v>
+        <v>726</v>
       </c>
       <c r="G191" s="111" t="n">
-        <v>8692</v>
+        <v>13310</v>
       </c>
       <c r="H191" s="111" t="n">
-        <v>1658</v>
+        <v>12850</v>
       </c>
       <c r="I191" s="111" t="n">
-        <v>7034</v>
+        <v>460</v>
       </c>
       <c r="J191" s="112" t="n">
-        <v>124.89</v>
+        <v>177</v>
       </c>
       <c r="K191" s="112" t="n">
-        <v>124.67</v>
-      </c>
-      <c r="L191" s="192">
+        <v>177</v>
+      </c>
+      <c r="L191" s="191">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -12284,31 +12288,31 @@
       <c r="C192" s="113" t="n"/>
       <c r="D192" s="110" t="inlineStr">
         <is>
-          <t>高力(8996)</t>
+          <t>聯電(2303)</t>
         </is>
       </c>
       <c r="E192" s="111" t="n">
-        <v>79</v>
+        <v>712</v>
       </c>
       <c r="F192" s="111" t="n">
-        <v>34</v>
+        <v>136</v>
       </c>
       <c r="G192" s="111" t="n">
-        <v>8310</v>
+        <v>8692</v>
       </c>
       <c r="H192" s="111" t="n">
-        <v>3634</v>
+        <v>1658</v>
       </c>
       <c r="I192" s="111" t="n">
-        <v>4676</v>
+        <v>7034</v>
       </c>
       <c r="J192" s="112" t="n">
-        <v>1051.9</v>
+        <v>122.08</v>
       </c>
       <c r="K192" s="112" t="n">
-        <v>1068.76</v>
-      </c>
-      <c r="L192" s="191">
+        <v>121.92</v>
+      </c>
+      <c r="L192" s="192">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -12319,29 +12323,29 @@
       <c r="C193" s="113" t="n"/>
       <c r="D193" s="110" t="inlineStr">
         <is>
-          <t>文曄(3036)</t>
+          <t>高力(8996)</t>
         </is>
       </c>
       <c r="E193" s="111" t="n">
-        <v>352</v>
+        <v>80</v>
       </c>
       <c r="F193" s="111" t="n">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="G193" s="111" t="n">
-        <v>7916</v>
+        <v>8310</v>
       </c>
       <c r="H193" s="111" t="n">
-        <v>1500</v>
+        <v>3634</v>
       </c>
       <c r="I193" s="111" t="n">
-        <v>6416</v>
+        <v>4676</v>
       </c>
       <c r="J193" s="112" t="n">
-        <v>224.89</v>
+        <v>1038.75</v>
       </c>
       <c r="K193" s="112" t="n">
-        <v>220.56</v>
+        <v>1038.23</v>
       </c>
       <c r="L193" s="192">
         <f>F193*(K193-J193)</f>
@@ -12354,31 +12358,31 @@
       <c r="C194" s="113" t="n"/>
       <c r="D194" s="110" t="inlineStr">
         <is>
-          <t>旺宏(2337)</t>
+          <t>文曄(3036)</t>
         </is>
       </c>
       <c r="E194" s="111" t="n">
-        <v>500</v>
+        <v>352</v>
       </c>
       <c r="F194" s="111" t="n">
-        <v>259</v>
+        <v>67</v>
       </c>
       <c r="G194" s="111" t="n">
-        <v>6135</v>
+        <v>7916</v>
       </c>
       <c r="H194" s="111" t="n">
-        <v>3188</v>
+        <v>1500</v>
       </c>
       <c r="I194" s="111" t="n">
-        <v>2947</v>
+        <v>6416</v>
       </c>
       <c r="J194" s="112" t="n">
-        <v>122.71</v>
+        <v>224.89</v>
       </c>
       <c r="K194" s="112" t="n">
-        <v>123.09</v>
-      </c>
-      <c r="L194" s="191">
+        <v>223.85</v>
+      </c>
+      <c r="L194" s="192">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -12389,29 +12393,29 @@
       <c r="C195" s="113" t="n"/>
       <c r="D195" s="110" t="inlineStr">
         <is>
-          <t>強茂(2481)</t>
+          <t>旺宏(2337)</t>
         </is>
       </c>
       <c r="E195" s="111" t="n">
-        <v>332</v>
+        <v>130</v>
       </c>
       <c r="F195" s="111" t="n">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="G195" s="111" t="n">
-        <v>4589</v>
+        <v>6135</v>
       </c>
       <c r="H195" s="111" t="n">
-        <v>245</v>
+        <v>3188</v>
       </c>
       <c r="I195" s="111" t="n">
-        <v>4344</v>
+        <v>2947</v>
       </c>
       <c r="J195" s="112" t="n">
-        <v>138.22</v>
+        <v>471.95</v>
       </c>
       <c r="K195" s="112" t="n">
-        <v>136.33</v>
+        <v>419.49</v>
       </c>
       <c r="L195" s="192">
         <f>F195*(K195-J195)</f>
@@ -12424,29 +12428,29 @@
       <c r="C196" s="113" t="n"/>
       <c r="D196" s="110" t="inlineStr">
         <is>
-          <t>華邦電(2344)</t>
+          <t>強茂(2481)</t>
         </is>
       </c>
       <c r="E196" s="111" t="n">
-        <v>185</v>
+        <v>342</v>
       </c>
       <c r="F196" s="111" t="n">
-        <v>164</v>
+        <v>18</v>
       </c>
       <c r="G196" s="111" t="n">
-        <v>3120</v>
+        <v>4589</v>
       </c>
       <c r="H196" s="111" t="n">
-        <v>2775</v>
+        <v>245</v>
       </c>
       <c r="I196" s="111" t="n">
-        <v>345</v>
+        <v>4344</v>
       </c>
       <c r="J196" s="112" t="n">
-        <v>168.64</v>
+        <v>134.18</v>
       </c>
       <c r="K196" s="112" t="n">
-        <v>169.2</v>
+        <v>136.33</v>
       </c>
       <c r="L196" s="191">
         <f>F196*(K196-J196)</f>
@@ -12459,29 +12463,29 @@
       <c r="C197" s="113" t="n"/>
       <c r="D197" s="110" t="inlineStr">
         <is>
-          <t>環球晶(6488)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E197" s="111" t="n">
-        <v>27</v>
+        <v>101</v>
       </c>
       <c r="F197" s="111" t="n">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="G197" s="111" t="n">
-        <v>2363</v>
+        <v>4494</v>
       </c>
       <c r="H197" s="111" t="n">
-        <v>1169</v>
+        <v>2448</v>
       </c>
       <c r="I197" s="111" t="n">
-        <v>1194</v>
+        <v>2046</v>
       </c>
       <c r="J197" s="112" t="n">
-        <v>875.22</v>
+        <v>445</v>
       </c>
       <c r="K197" s="112" t="n">
-        <v>899.38</v>
+        <v>445</v>
       </c>
       <c r="L197" s="191">
         <f>F197*(K197-J197)</f>
@@ -12494,29 +12498,29 @@
       <c r="C198" s="113" t="n"/>
       <c r="D198" s="110" t="inlineStr">
         <is>
-          <t>群創(3481)</t>
+          <t>華邦電(2344)</t>
         </is>
       </c>
       <c r="E198" s="111" t="n">
-        <v>403</v>
+        <v>185</v>
       </c>
       <c r="F198" s="111" t="n">
-        <v>367</v>
+        <v>164</v>
       </c>
       <c r="G198" s="111" t="n">
-        <v>1926</v>
+        <v>3120</v>
       </c>
       <c r="H198" s="111" t="n">
-        <v>1754</v>
+        <v>2775</v>
       </c>
       <c r="I198" s="111" t="n">
-        <v>172</v>
+        <v>345</v>
       </c>
       <c r="J198" s="112" t="n">
-        <v>47.8</v>
+        <v>168.64</v>
       </c>
       <c r="K198" s="112" t="n">
-        <v>47.8</v>
+        <v>169.2</v>
       </c>
       <c r="L198" s="191">
         <f>F198*(K198-J198)</f>
@@ -12529,29 +12533,29 @@
       <c r="C199" s="113" t="n"/>
       <c r="D199" s="110" t="inlineStr">
         <is>
-          <t>力成(6239)</t>
+          <t>環球晶(6488)</t>
         </is>
       </c>
       <c r="E199" s="111" t="n">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="F199" s="111" t="n">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="G199" s="111" t="n">
-        <v>1909</v>
+        <v>2363</v>
       </c>
       <c r="H199" s="111" t="n">
-        <v>1678</v>
+        <v>1169</v>
       </c>
       <c r="I199" s="111" t="n">
-        <v>231</v>
+        <v>1194</v>
       </c>
       <c r="J199" s="112" t="n">
-        <v>258</v>
+        <v>875.22</v>
       </c>
       <c r="K199" s="112" t="n">
-        <v>258.12</v>
+        <v>899.38</v>
       </c>
       <c r="L199" s="191">
         <f>F199*(K199-J199)</f>
@@ -23181,7 +23185,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="177" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-08-05 15:41 | 0/19 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-08-05 16:33 | 0/19 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-08-06 01:24
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -23,7 +23,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="18">
+  <numFmts count="19">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-64/5d-140)&quot;;-0&quot; 億 (昨-64/5d-140)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +122億 &quot;&quot;(昨5/5d9)&quot;"/>
@@ -42,6 +42,7 @@
     <numFmt numFmtId="179" formatCode="0&quot; 檔 +63億 &quot;&quot;(昨9/5d8)&quot;"/>
     <numFmt numFmtId="180" formatCode="0.0%&quot; 市-482億 &quot;&quot;(昨18/5d18)&quot;"/>
     <numFmt numFmtId="181" formatCode="0.0%&quot; 市-475億 &quot;&quot;(昨18/5d18)&quot;"/>
+    <numFmt numFmtId="182" formatCode="0.0%&quot; 市-477億 &quot;&quot;(昨18/5d18)&quot;"/>
   </numFmts>
   <fonts count="39">
     <font>
@@ -269,7 +270,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="48">
+  <fills count="49">
     <fill>
       <patternFill/>
     </fill>
@@ -508,6 +509,12 @@
         <fgColor rgb="FFFBBF24"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -521,7 +528,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="205">
+  <cellXfs count="211">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -985,6 +992,24 @@
     <xf numFmtId="181" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="182" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="4" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="5" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1070,12 +1095,12 @@
     <comment ref="D15" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「張濬安(航海王)」獨佔比 60.3%
+領頭大戶「張濬安(航海王)」獨佔比 60.9%
   • 領頭金額 136,742 萬
-  • 合計淨買 226,692 萬
+  • 合計淨買 224,645 萬
   • 大戶數 10 位 (名義共識)
 判讀: 名義 10 位大戶共識,
-實質 1 人下注佔 60%,
+實質 1 人下注佔 61%,
 剩餘 9 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1444,7 +1469,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 📌 一般共識 2408 / 2303 / 2368 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 除權息 6 檔: 00400A, 1437, 1519 ...  |  訊號: 強偏多 (Q5 95%, hot=3)</t>
+          <t>💡 📌 一般共識 2408 / 2303 / 2368 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開: 今日無除權息+處置股  |  訊號: 強偏多 (Q5 95%, hot=3)</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
@@ -1605,7 +1630,7 @@
         </is>
       </c>
       <c r="J15" s="18" t="n">
-        <v>58107</v>
+        <v>56060</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1619,7 +1644,7 @@
         <v>7</v>
       </c>
       <c r="N15" s="17" t="n">
-        <v>226692</v>
+        <v>224645</v>
       </c>
     </row>
     <row r="16">
@@ -1997,7 +2022,7 @@
         <v>11</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
@@ -2005,7 +2030,7 @@
         </is>
       </c>
       <c r="H23" s="17" t="n">
-        <v>4888</v>
+        <v>5060</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -2027,7 +2052,7 @@
         <v>8</v>
       </c>
       <c r="N23" s="17" t="n">
-        <v>18830</v>
+        <v>19002</v>
       </c>
     </row>
     <row r="24">
@@ -2150,7 +2175,7 @@
         <v>10</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G26" s="16" t="inlineStr">
         <is>
@@ -2180,7 +2205,7 @@
         <v>7</v>
       </c>
       <c r="N26" s="17" t="n">
-        <v>7848</v>
+        <v>7730</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
@@ -2205,7 +2230,7 @@
         </is>
       </c>
       <c r="G29" s="200" t="n">
-        <v>-183.99805</v>
+        <v>-187.38063</v>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
@@ -2222,8 +2247,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G30" s="204" t="n">
-        <v>0.1595358900128013</v>
+      <c r="G30" s="205" t="n">
+        <v>0.159159685079513</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
@@ -2306,7 +2331,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>35.5%</t>
+          <t>35.6%</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2334,11 +2359,11 @@
         </is>
       </c>
       <c r="D37" s="33" t="n">
-        <v>1509116</v>
+        <v>1489607</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>27.0%</t>
+          <t>26.8%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2350,7 +2375,7 @@
         </is>
       </c>
       <c r="H37" s="33" t="n">
-        <v>226692</v>
+        <v>224645</v>
       </c>
       <c r="I37" s="184" t="n">
         <v>0.0206</v>
@@ -2742,18 +2767,18 @@
       </c>
       <c r="C58" s="58" t="inlineStr">
         <is>
-          <t>1303</t>
+          <t>2383</t>
         </is>
       </c>
       <c r="D58" s="58" t="n">
         <v>4</v>
       </c>
       <c r="E58" s="58" t="n">
-        <v>232315</v>
+        <v>230495</v>
       </c>
       <c r="F58" s="58" t="inlineStr">
         <is>
-          <t>陳族元 連續 4 天加碼 1303 (累計 232,315 萬)</t>
+          <t>陳族元 連續 4 天加碼 2383 (累計 230,495 萬)</t>
         </is>
       </c>
     </row>
@@ -2765,18 +2790,18 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2383</t>
+          <t>3653</t>
         </is>
       </c>
       <c r="D59" t="n">
         <v>4</v>
       </c>
       <c r="E59" t="n">
-        <v>230495</v>
+        <v>228922</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>陳族元 連續 4 天加碼 2383 (累計 230,495 萬)</t>
+          <t>陳族元 連續 4 天加碼 3653 (累計 228,922 萬)</t>
         </is>
       </c>
     </row>
@@ -2788,18 +2813,18 @@
       </c>
       <c r="C60" s="58" t="inlineStr">
         <is>
-          <t>3653</t>
+          <t>1303</t>
         </is>
       </c>
       <c r="D60" s="58" t="n">
         <v>4</v>
       </c>
       <c r="E60" s="58" t="n">
-        <v>228922</v>
+        <v>219005</v>
       </c>
       <c r="F60" s="58" t="inlineStr">
         <is>
-          <t>陳族元 連續 4 天加碼 3653 (累計 228,922 萬)</t>
+          <t>陳族元 連續 4 天加碼 1303 (累計 219,005 萬)</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2972,7 @@
         </is>
       </c>
       <c r="C67" s="33" t="n">
-        <v>1389992</v>
+        <v>1371660</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -2974,7 +2999,7 @@
         <v>124487</v>
       </c>
       <c r="J67" s="185" t="n">
-        <v>0.3231317667636168</v>
+        <v>0.3274504853571938</v>
       </c>
     </row>
     <row r="68">
@@ -3387,7 +3412,7 @@
     <row r="80" ht="22" customHeight="1">
       <c r="B80" s="54" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20260805)</t>
+          <t>▍ G. 注意股 (資料日 20260806)</t>
         </is>
       </c>
     </row>
@@ -3779,7 +3804,7 @@
     <row r="102" ht="22" customHeight="1">
       <c r="B102" s="65" t="inlineStr">
         <is>
-          <t>▍ I. 未來 30 天除權息 (有效 104 檔, 已剔除過期)</t>
+          <t>▍ I. 未來 30 天除權息 (有效 99 檔, 已剔除過期)</t>
         </is>
       </c>
     </row>
@@ -3813,17 +3838,17 @@
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>20260805</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>00400A</t>
+          <t>1419</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>主動國泰動能高息</t>
+          <t>新紡</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -3832,23 +3857,23 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>0.12</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="105">
       <c r="B105" s="58" t="inlineStr">
         <is>
-          <t>20260805</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C105" s="58" t="inlineStr">
         <is>
-          <t>1437</t>
+          <t>1439</t>
         </is>
       </c>
       <c r="D105" s="58" t="inlineStr">
         <is>
-          <t>勤益控</t>
+          <t>雋揚</t>
         </is>
       </c>
       <c r="E105" s="58" t="inlineStr">
@@ -3857,48 +3882,48 @@
         </is>
       </c>
       <c r="F105" s="58" t="n">
-        <v>0.481191</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="106">
       <c r="B106" t="inlineStr">
         <is>
-          <t>20260805</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>1519</t>
+          <t>1713</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>華城</t>
+          <t>國化</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>權息</t>
+          <t>息</t>
         </is>
       </c>
       <c r="F106" t="n">
-        <v>11</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="107">
       <c r="B107" s="58" t="inlineStr">
         <is>
-          <t>20260805</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C107" s="58" t="inlineStr">
         <is>
-          <t>2427</t>
+          <t>2375</t>
         </is>
       </c>
       <c r="D107" s="58" t="inlineStr">
         <is>
-          <t>三商電</t>
+          <t>凱美</t>
         </is>
       </c>
       <c r="E107" s="58" t="inlineStr">
@@ -3907,48 +3932,48 @@
         </is>
       </c>
       <c r="F107" s="58" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t>20260805</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2801</t>
+          <t>2762</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>彰銀</t>
+          <t>世界健身-KY</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>權息</t>
+          <t>息</t>
         </is>
       </c>
       <c r="F108" t="n">
-        <v>0.8</v>
+        <v>3.636991</v>
       </c>
     </row>
     <row r="109">
       <c r="B109" s="58" t="inlineStr">
         <is>
-          <t>20260805</t>
+          <t>20260806</t>
         </is>
       </c>
       <c r="C109" s="58" t="inlineStr">
         <is>
-          <t>6201</t>
+          <t>3003</t>
         </is>
       </c>
       <c r="D109" s="58" t="inlineStr">
         <is>
-          <t>亞弘電</t>
+          <t>健和興</t>
         </is>
       </c>
       <c r="E109" s="58" t="inlineStr">
@@ -3957,7 +3982,7 @@
         </is>
       </c>
       <c r="F109" s="58" t="n">
-        <v>3.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110">
@@ -3968,12 +3993,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>1419</t>
+          <t>3033</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>新紡</t>
+          <t>威健</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -3982,7 +4007,7 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>1.8</v>
+        <v>1.919856</v>
       </c>
     </row>
     <row r="111">
@@ -3993,12 +4018,12 @@
       </c>
       <c r="C111" s="58" t="inlineStr">
         <is>
-          <t>1439</t>
+          <t>3376</t>
         </is>
       </c>
       <c r="D111" s="58" t="inlineStr">
         <is>
-          <t>雋揚</t>
+          <t>新日興</t>
         </is>
       </c>
       <c r="E111" s="58" t="inlineStr">
@@ -4007,7 +4032,7 @@
         </is>
       </c>
       <c r="F111" s="58" t="n">
-        <v>0.5</v>
+        <v>3.999665</v>
       </c>
     </row>
     <row r="112">
@@ -4018,12 +4043,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>1713</t>
+          <t>5288</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>國化</t>
+          <t>豐祥-KY</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -4032,7 +4057,7 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>3.1</v>
+        <v>6.502918</v>
       </c>
     </row>
     <row r="113">
@@ -4043,12 +4068,12 @@
       </c>
       <c r="C113" s="58" t="inlineStr">
         <is>
-          <t>2375</t>
+          <t>5525</t>
         </is>
       </c>
       <c r="D113" s="58" t="inlineStr">
         <is>
-          <t>凱美</t>
+          <t>順天</t>
         </is>
       </c>
       <c r="E113" s="58" t="inlineStr">
@@ -4068,12 +4093,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2762</t>
+          <t>9914</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>世界健身-KY</t>
+          <t>美利達</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -4082,23 +4107,23 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>3.636991</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="115">
       <c r="B115" s="58" t="inlineStr">
         <is>
-          <t>20260806</t>
+          <t>20260807</t>
         </is>
       </c>
       <c r="C115" s="58" t="inlineStr">
         <is>
-          <t>3003</t>
+          <t>1210</t>
         </is>
       </c>
       <c r="D115" s="58" t="inlineStr">
         <is>
-          <t>健和興</t>
+          <t>大成</t>
         </is>
       </c>
       <c r="E115" s="58" t="inlineStr">
@@ -4107,23 +4132,23 @@
         </is>
       </c>
       <c r="F115" s="58" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="116">
       <c r="B116" t="inlineStr">
         <is>
-          <t>20260806</t>
+          <t>20260807</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>3033</t>
+          <t>6491</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>威健</t>
+          <t>晶碩</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -4132,23 +4157,23 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>1.919856</v>
+        <v>10.00513</v>
       </c>
     </row>
     <row r="117">
       <c r="B117" s="58" t="inlineStr">
         <is>
-          <t>20260806</t>
+          <t>20260810</t>
         </is>
       </c>
       <c r="C117" s="58" t="inlineStr">
         <is>
-          <t>3376</t>
+          <t>2520</t>
         </is>
       </c>
       <c r="D117" s="58" t="inlineStr">
         <is>
-          <t>新日興</t>
+          <t>冠德</t>
         </is>
       </c>
       <c r="E117" s="58" t="inlineStr">
@@ -4157,23 +4182,23 @@
         </is>
       </c>
       <c r="F117" s="58" t="n">
-        <v>3.999665</v>
+        <v>1.615933</v>
       </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t>20260806</t>
+          <t>20260810</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>5288</t>
+          <t>2540</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>豐祥-KY</t>
+          <t>愛山林</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -4182,7 +4207,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>6.502918</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -4497,9 +4522,9 @@
       </c>
     </row>
     <row r="32">
-      <c r="C32" s="69" t="inlineStr">
-        <is>
-          <t>除權息 6 檔 (00400A / 1437 / 1519 ...)</t>
+      <c r="C32" s="71" t="inlineStr">
+        <is>
+          <t>今日無除權息</t>
         </is>
       </c>
     </row>
@@ -4520,7 +4545,7 @@
     <row r="36" ht="22" customHeight="1">
       <c r="C36" s="198" t="inlineStr">
         <is>
-          <t>-184 億 淨買</t>
+          <t>-187 億 淨買</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4669,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="B3" s="76" t="inlineStr">
         <is>
-          <t>大牌分析師 近 4/4 交易日出手 183 次 (138 檔), 風格分布: 隔日沖近似 25% / 當沖 17% / 留倉 58%, 漲停命中 9% (其中 🔒鎖漲停 7%), 前 5 大集中 28%, ⚠️ 處置股部位 2% (5 檔)。 主軸: 高頻交易。</t>
+          <t>大牌分析師 近 4/4 交易日出手 183 次 (138 檔), 風格分布: 隔日沖近似 25% / 當沖 17% / 留倉 58%, 漲停命中 9% (其中 🔒鎖漲停 7%), 前 5 大集中 28%, ⚠️ 處置股部位 2% (6 檔)。 主軸: 高頻交易。</t>
         </is>
       </c>
     </row>
@@ -5030,7 +5055,7 @@
       <c r="C1" s="80" t="n"/>
       <c r="D1" s="81" t="inlineStr">
         <is>
-          <t>⚠️ 本 Excel 無 top-buyer highlight — histock 分點榜無資料 (可能個股冷門) (histock: 19 試, 0 success)</t>
+          <t>⚠️ 部分 top-buyer highlight 缺 (histock: 2/19 = 10% success | stale=0 http_err=0 no_data=17)</t>
         </is>
       </c>
       <c r="E1" s="82" t="n"/>
@@ -12253,31 +12278,31 @@
       <c r="C191" s="113" t="n"/>
       <c r="D191" s="110" t="inlineStr">
         <is>
-          <t>南亞(1303)</t>
+          <t>聯電(2303)</t>
         </is>
       </c>
       <c r="E191" s="111" t="n">
-        <v>752</v>
+        <v>696</v>
       </c>
       <c r="F191" s="111" t="n">
-        <v>726</v>
+        <v>133</v>
       </c>
       <c r="G191" s="111" t="n">
-        <v>13310</v>
+        <v>8692</v>
       </c>
       <c r="H191" s="111" t="n">
-        <v>12850</v>
+        <v>1658</v>
       </c>
       <c r="I191" s="111" t="n">
-        <v>460</v>
+        <v>7034</v>
       </c>
       <c r="J191" s="112" t="n">
-        <v>177</v>
+        <v>124.89</v>
       </c>
       <c r="K191" s="112" t="n">
-        <v>177</v>
-      </c>
-      <c r="L191" s="191">
+        <v>124.67</v>
+      </c>
+      <c r="L191" s="192">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -12288,31 +12313,31 @@
       <c r="C192" s="113" t="n"/>
       <c r="D192" s="110" t="inlineStr">
         <is>
-          <t>聯電(2303)</t>
+          <t>高力(8996)</t>
         </is>
       </c>
       <c r="E192" s="111" t="n">
-        <v>712</v>
+        <v>79</v>
       </c>
       <c r="F192" s="111" t="n">
-        <v>136</v>
+        <v>34</v>
       </c>
       <c r="G192" s="111" t="n">
-        <v>8692</v>
+        <v>8310</v>
       </c>
       <c r="H192" s="111" t="n">
-        <v>1658</v>
+        <v>3634</v>
       </c>
       <c r="I192" s="111" t="n">
-        <v>7034</v>
+        <v>4676</v>
       </c>
       <c r="J192" s="112" t="n">
-        <v>122.08</v>
+        <v>1051.9</v>
       </c>
       <c r="K192" s="112" t="n">
-        <v>121.92</v>
-      </c>
-      <c r="L192" s="192">
+        <v>1068.76</v>
+      </c>
+      <c r="L192" s="191">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -12323,29 +12348,29 @@
       <c r="C193" s="113" t="n"/>
       <c r="D193" s="110" t="inlineStr">
         <is>
-          <t>高力(8996)</t>
+          <t>文曄(3036)</t>
         </is>
       </c>
       <c r="E193" s="111" t="n">
-        <v>80</v>
+        <v>352</v>
       </c>
       <c r="F193" s="111" t="n">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="G193" s="111" t="n">
-        <v>8310</v>
+        <v>7916</v>
       </c>
       <c r="H193" s="111" t="n">
-        <v>3634</v>
+        <v>1500</v>
       </c>
       <c r="I193" s="111" t="n">
-        <v>4676</v>
+        <v>6416</v>
       </c>
       <c r="J193" s="112" t="n">
-        <v>1038.75</v>
+        <v>224.89</v>
       </c>
       <c r="K193" s="112" t="n">
-        <v>1038.23</v>
+        <v>220.56</v>
       </c>
       <c r="L193" s="192">
         <f>F193*(K193-J193)</f>
@@ -12358,31 +12383,31 @@
       <c r="C194" s="113" t="n"/>
       <c r="D194" s="110" t="inlineStr">
         <is>
-          <t>文曄(3036)</t>
+          <t>旺宏(2337)</t>
         </is>
       </c>
       <c r="E194" s="111" t="n">
-        <v>352</v>
+        <v>500</v>
       </c>
       <c r="F194" s="111" t="n">
-        <v>67</v>
+        <v>259</v>
       </c>
       <c r="G194" s="111" t="n">
-        <v>7916</v>
+        <v>6135</v>
       </c>
       <c r="H194" s="111" t="n">
-        <v>1500</v>
+        <v>3188</v>
       </c>
       <c r="I194" s="111" t="n">
-        <v>6416</v>
+        <v>2947</v>
       </c>
       <c r="J194" s="112" t="n">
-        <v>224.89</v>
+        <v>122.71</v>
       </c>
       <c r="K194" s="112" t="n">
-        <v>223.85</v>
-      </c>
-      <c r="L194" s="192">
+        <v>123.09</v>
+      </c>
+      <c r="L194" s="191">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -12393,29 +12418,29 @@
       <c r="C195" s="113" t="n"/>
       <c r="D195" s="110" t="inlineStr">
         <is>
-          <t>旺宏(2337)</t>
+          <t>強茂(2481)</t>
         </is>
       </c>
       <c r="E195" s="111" t="n">
-        <v>130</v>
+        <v>332</v>
       </c>
       <c r="F195" s="111" t="n">
-        <v>76</v>
+        <v>18</v>
       </c>
       <c r="G195" s="111" t="n">
-        <v>6135</v>
+        <v>4589</v>
       </c>
       <c r="H195" s="111" t="n">
-        <v>3188</v>
+        <v>245</v>
       </c>
       <c r="I195" s="111" t="n">
-        <v>2947</v>
+        <v>4344</v>
       </c>
       <c r="J195" s="112" t="n">
-        <v>471.95</v>
+        <v>138.22</v>
       </c>
       <c r="K195" s="112" t="n">
-        <v>419.49</v>
+        <v>136.33</v>
       </c>
       <c r="L195" s="192">
         <f>F195*(K195-J195)</f>
@@ -12428,29 +12453,29 @@
       <c r="C196" s="113" t="n"/>
       <c r="D196" s="110" t="inlineStr">
         <is>
-          <t>強茂(2481)</t>
+          <t>華邦電(2344)</t>
         </is>
       </c>
       <c r="E196" s="111" t="n">
-        <v>342</v>
+        <v>185</v>
       </c>
       <c r="F196" s="111" t="n">
-        <v>18</v>
+        <v>164</v>
       </c>
       <c r="G196" s="111" t="n">
-        <v>4589</v>
+        <v>3120</v>
       </c>
       <c r="H196" s="111" t="n">
-        <v>245</v>
+        <v>2775</v>
       </c>
       <c r="I196" s="111" t="n">
-        <v>4344</v>
+        <v>345</v>
       </c>
       <c r="J196" s="112" t="n">
-        <v>134.18</v>
+        <v>168.64</v>
       </c>
       <c r="K196" s="112" t="n">
-        <v>136.33</v>
+        <v>169.2</v>
       </c>
       <c r="L196" s="191">
         <f>F196*(K196-J196)</f>
@@ -12463,29 +12488,29 @@
       <c r="C197" s="113" t="n"/>
       <c r="D197" s="110" t="inlineStr">
         <is>
-          <t>南亞科(2408)</t>
+          <t>環球晶(6488)</t>
         </is>
       </c>
       <c r="E197" s="111" t="n">
-        <v>101</v>
+        <v>27</v>
       </c>
       <c r="F197" s="111" t="n">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="G197" s="111" t="n">
-        <v>4494</v>
+        <v>2363</v>
       </c>
       <c r="H197" s="111" t="n">
-        <v>2448</v>
+        <v>1169</v>
       </c>
       <c r="I197" s="111" t="n">
-        <v>2046</v>
+        <v>1194</v>
       </c>
       <c r="J197" s="112" t="n">
-        <v>445</v>
+        <v>875.22</v>
       </c>
       <c r="K197" s="112" t="n">
-        <v>445</v>
+        <v>899.38</v>
       </c>
       <c r="L197" s="191">
         <f>F197*(K197-J197)</f>
@@ -12498,29 +12523,29 @@
       <c r="C198" s="113" t="n"/>
       <c r="D198" s="110" t="inlineStr">
         <is>
-          <t>華邦電(2344)</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E198" s="111" t="n">
-        <v>185</v>
+        <v>403</v>
       </c>
       <c r="F198" s="111" t="n">
-        <v>164</v>
+        <v>367</v>
       </c>
       <c r="G198" s="111" t="n">
-        <v>3120</v>
+        <v>1926</v>
       </c>
       <c r="H198" s="111" t="n">
-        <v>2775</v>
+        <v>1754</v>
       </c>
       <c r="I198" s="111" t="n">
-        <v>345</v>
+        <v>172</v>
       </c>
       <c r="J198" s="112" t="n">
-        <v>168.64</v>
+        <v>47.8</v>
       </c>
       <c r="K198" s="112" t="n">
-        <v>169.2</v>
+        <v>47.8</v>
       </c>
       <c r="L198" s="191">
         <f>F198*(K198-J198)</f>
@@ -12533,29 +12558,29 @@
       <c r="C199" s="113" t="n"/>
       <c r="D199" s="110" t="inlineStr">
         <is>
-          <t>環球晶(6488)</t>
+          <t>力成(6239)</t>
         </is>
       </c>
       <c r="E199" s="111" t="n">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="F199" s="111" t="n">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="G199" s="111" t="n">
-        <v>2363</v>
+        <v>1909</v>
       </c>
       <c r="H199" s="111" t="n">
-        <v>1169</v>
+        <v>1678</v>
       </c>
       <c r="I199" s="111" t="n">
-        <v>1194</v>
+        <v>231</v>
       </c>
       <c r="J199" s="112" t="n">
-        <v>875.22</v>
+        <v>258</v>
       </c>
       <c r="K199" s="112" t="n">
-        <v>899.38</v>
+        <v>258.12</v>
       </c>
       <c r="L199" s="191">
         <f>F199*(K199-J199)</f>
@@ -23185,7 +23210,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="177" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-08-05 16:33 | 0/19 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-08-05 17:24 | 2/19 success</t>
         </is>
       </c>
     </row>

</xml_diff>